<commit_message>
Rename database tables for cleaning workflow
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/basic-design.xlsx
+++ b/docs/basic-design.xlsx
@@ -256,7 +256,7 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">社員マスタと掃除エリアマスタをもとに、翌週5日分の掃除当番をランダムに抽選・登録し、一覧表示する Web アプリケーション。</t>
+          <t xml:space="preserve">社員 (person) と掃除タスク (task) をもとに、翌週5日分の掃除当番をランダムに抽選・登録し、一覧表示する Web アプリケーション。</t>
         </is>
       </c>
     </row>
@@ -1146,7 +1146,7 @@
       </c>
       <c r="C85" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">GORM を使った DB アクセス。employee / area / duty の3つ</t>
+          <t xml:space="preserve">GORM を使った DB アクセス。person / task / lottery_result に対応</t>
         </is>
       </c>
     </row>
@@ -1163,7 +1163,7 @@
       </c>
       <c r="C86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">GORM モデル (Employee / Area / Duty) と API 応答用の DutyView</t>
+          <t xml:space="preserve">GORM モデル (Employee / Area / Duty) と API 応答用の DutyView。Area は task の互換APIモデル</t>
         </is>
       </c>
     </row>
@@ -1368,21 +1368,21 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">・employees から active = 1 の社員 ID を全件取得する。</t>
+          <t xml:space="preserve">・person から active = 1 の社員 ID を全件取得する。</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">・areas から全エリア ID を取得する。</t>
+          <t xml:space="preserve">・task から全掃除タスク ID を取得する。</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">・いずれかが空の場合はエラー (employees or areas is empty) とし、HTTP 400 を返す。</t>
+          <t xml:space="preserve">・いずれかが空の場合はエラー (person or task is empty) とし、HTTP 400 を返す。</t>
         </is>
       </c>
     </row>

</xml_diff>